<commit_message>
Phase 2 update: apply operator-review spec changes
- docs/SPEC.md replaced with the reviewed version (section 15, G9.1-G9.12)
- Eyewear minimum investment now 30 / 20 / 15 lakh; status labels per SPEC 6.1
- Fixture: re-banded rows for the new minimums and the 15.5 offer order; new cases
  for owned space at an existing-store pin (APP-034), 3 months + before Diwali (APP-026),
  provisional win while on hold (APP-035), similar names Ravi Kumar / Ravi K (APP-036/037);
  rows moved off the example territory's pins
- Heuristic signals return exact matched text as evidence; note-based issues carry it
- Data-quality report warns when the skipped example territory covers an applicant (G9.8)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sampleWorkbook.xlsx
+++ b/data/sampleWorkbook.xlsx
@@ -706,7 +706,7 @@
         <v>560102</v>
       </c>
       <c r="F8">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G8">
         <v>6</v>
@@ -882,7 +882,7 @@
         <v>560043</v>
       </c>
       <c r="F12">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G12">
         <v>2</v>
@@ -979,7 +979,7 @@
         <v>Runs a bakery</v>
       </c>
       <c r="I14" t="str">
-        <v>Owned</v>
+        <v>Rented</v>
       </c>
       <c r="J14">
         <v>500</v>
@@ -1052,7 +1052,7 @@
         <v>560029</v>
       </c>
       <c r="F16">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G16">
         <v>2</v>
@@ -1096,7 +1096,7 @@
         <v>560029</v>
       </c>
       <c r="F17">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G17">
         <v>2</v>
@@ -1272,7 +1272,7 @@
         <v>572102</v>
       </c>
       <c r="F21">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -1316,7 +1316,7 @@
         <v>560037</v>
       </c>
       <c r="F22">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="G22">
         <v>5</v>
@@ -1530,7 +1530,7 @@
         <v>560036</v>
       </c>
       <c r="F27">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G27">
         <v>3</v>
@@ -1571,7 +1571,7 @@
         <v>Karnataka</v>
       </c>
       <c r="E28">
-        <v>570020</v>
+        <v>570023</v>
       </c>
       <c r="F28">
         <v>38</v>
@@ -1615,7 +1615,7 @@
         <v>Karnataka</v>
       </c>
       <c r="E29">
-        <v>570008</v>
+        <v>570020</v>
       </c>
       <c r="F29">
         <v>45</v>
@@ -1630,7 +1630,7 @@
         <v>Not yet identified</v>
       </c>
       <c r="L29">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M29" t="str">
         <v>Kannada</v>
@@ -1982,6 +1982,182 @@
         <v>Kannada</v>
       </c>
       <c r="N37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>APP-034</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Prakash Hegde</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Mysuru</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="E38">
+        <v>570009</v>
+      </c>
+      <c r="F38">
+        <v>40</v>
+      </c>
+      <c r="G38">
+        <v>6</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Footwear retail</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Owned</v>
+      </c>
+      <c r="J38">
+        <v>600</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Ground</v>
+      </c>
+      <c r="L38">
+        <v>4</v>
+      </c>
+      <c r="M38" t="str">
+        <v>Kannada</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Own a shop in Saraswathipuram</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>APP-035</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Lokesh Reddy</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Bengaluru</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="E39">
+        <v>560037</v>
+      </c>
+      <c r="F39">
+        <v>60</v>
+      </c>
+      <c r="G39">
+        <v>6</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Electronics retail</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Rented</v>
+      </c>
+      <c r="J39">
+        <v>600</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Ground</v>
+      </c>
+      <c r="L39">
+        <v>4</v>
+      </c>
+      <c r="M39" t="str">
+        <v>English</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Shop on the ground floor with the first floor used for storage</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>APP-036</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Ravi Kumar</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Davanagere</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="E40">
+        <v>577002</v>
+      </c>
+      <c r="F40">
+        <v>30</v>
+      </c>
+      <c r="G40">
+        <v>4</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Footwear retail</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Rented</v>
+      </c>
+      <c r="J40">
+        <v>450</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Ground</v>
+      </c>
+      <c r="L40">
+        <v>4</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Kannada</v>
+      </c>
+      <c r="N40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>APP-037</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Ravi K</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Mangaluru</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="E41">
+        <v>575003</v>
+      </c>
+      <c r="F41">
+        <v>28</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Mobile accessories</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Rented</v>
+      </c>
+      <c r="J41">
+        <v>400</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Ground</v>
+      </c>
+      <c r="L41">
+        <v>4</v>
+      </c>
+      <c r="M41" t="str">
+        <v>English</v>
+      </c>
+      <c r="N41" t="str">
         <v/>
       </c>
     </row>
@@ -2098,7 +2274,7 @@
         <v>Karnataka</v>
       </c>
       <c r="D5" t="str">
-        <v>560038, 560037, 560048, 560036, 560093, 560047</v>
+        <v>560038, 560037, 560048, 560036, 560093, 560047, 560017</v>
       </c>
       <c r="E5" t="str">
         <v>Tier 1</v>
@@ -2144,13 +2320,13 @@
         <v>Karnataka</v>
       </c>
       <c r="D7" t="str">
-        <v>570005, 570008, 570009, 570010, 570015, 570020</v>
+        <v>570004, 570005, 570009, 570010, 570015, 570020</v>
       </c>
       <c r="E7" t="str">
         <v>Tier 1</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G7" t="str">
         <v>High</v>

</xml_diff>